<commit_message>
Fix ZIRAAT commission extraction - use correct regex pattern
Previous regex captured trailing commas, breaking parsing. Fixed to only
capture number with decimal: ([0-9]+[,\.][0-9]+)

Correct total: 268,375.47 TL (not 6,642.55 TL)

01-10.07: 94,157.61 TL
11-20.07: 76,196.00 TL
21-31.07: 98,021.86 TL

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013XirDLHEgVkT9Fvb27rTq6
</commit_message>
<xml_diff>
--- a/ZİRAAT-KOMİSYON-Temmuz2026.xlsx
+++ b/ZİRAAT-KOMİSYON-Temmuz2026.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>6642.55</v>
+        <v>268375.47</v>
       </c>
     </row>
     <row r="3">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>178.94</v>
+        <v>9623.060000000001</v>
       </c>
     </row>
     <row r="6">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>392.26</v>
+        <v>8669.419999999998</v>
       </c>
     </row>
     <row r="7">
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>170.62</v>
+        <v>6183.459999999998</v>
       </c>
     </row>
     <row r="8">
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>882.0999999999998</v>
+        <v>31608.62999999998</v>
       </c>
     </row>
     <row r="9">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>210.74</v>
+        <v>8172.870000000001</v>
       </c>
     </row>
     <row r="10">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>151.66</v>
+        <v>8748.59</v>
       </c>
     </row>
     <row r="11">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>133.81</v>
+        <v>11597.95</v>
       </c>
     </row>
     <row r="12">
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>313.86</v>
+        <v>9553.629999999999</v>
       </c>
     </row>
     <row r="13">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>2433.99</v>
+        <v>94157.60999999999</v>
       </c>
     </row>
     <row r="15">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>548.41</v>
+        <v>29136.6</v>
       </c>
     </row>
     <row r="17">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>122.76</v>
+        <v>5402</v>
       </c>
     </row>
     <row r="18">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>424.83</v>
+        <v>10899.41</v>
       </c>
     </row>
     <row r="19">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>252.86</v>
+        <v>7979.389999999999</v>
       </c>
     </row>
     <row r="20">
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>666.6799999999999</v>
+        <v>22778.60000000001</v>
       </c>
     </row>
     <row r="21">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>2015.54</v>
+        <v>76196</v>
       </c>
     </row>
     <row r="23">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>55.76000000000001</v>
+        <v>5622.52</v>
       </c>
     </row>
     <row r="25">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>98.94</v>
+        <v>9385.91</v>
       </c>
     </row>
     <row r="26">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>93.55000000000001</v>
+        <v>6850.969999999999</v>
       </c>
     </row>
     <row r="27">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>92.56</v>
+        <v>8356.820000000003</v>
       </c>
     </row>
     <row r="28">
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>858.1999999999999</v>
+        <v>29335.50000000001</v>
       </c>
     </row>
     <row r="29">
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>106.52</v>
+        <v>6715.990000000001</v>
       </c>
     </row>
     <row r="30">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>108.02</v>
+        <v>8493.5</v>
       </c>
     </row>
     <row r="31">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>218.83</v>
+        <v>9704.750000000002</v>
       </c>
     </row>
     <row r="32">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>560.64</v>
+        <v>13555.9</v>
       </c>
     </row>
     <row r="33">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>2193.02</v>
+        <v>98021.86000000002</v>
       </c>
     </row>
     <row r="35">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="B35" s="10" t="n">
-        <v>6642.55</v>
+        <v>268375.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix ZIRAAT commission extraction - only count POS SATIŞ transactions
Previous version counted all Komisyon rows including accounting entries.
Correct filter is 'POS SATIŞ' transactions only, like AKBANK 'KS:' pattern.

Correct total: 5,811.55 TL (not 268,375.47 TL)

01-10.07: 1,825.99 TL
11-20.07: 1,792.54 TL
21-31.07: 2,193.02 TL

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013XirDLHEgVkT9Fvb27rTq6
</commit_message>
<xml_diff>
--- a/ZİRAAT-KOMİSYON-Temmuz2026.xlsx
+++ b/ZİRAAT-KOMİSYON-Temmuz2026.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>268375.47</v>
+        <v>5811.55</v>
       </c>
     </row>
     <row r="3">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>9623.060000000001</v>
+        <v>178.94</v>
       </c>
     </row>
     <row r="6">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>8669.419999999998</v>
+        <v>232.26</v>
       </c>
     </row>
     <row r="7">
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>6183.459999999998</v>
+        <v>170.62</v>
       </c>
     </row>
     <row r="8">
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>31608.62999999998</v>
+        <v>440.1</v>
       </c>
     </row>
     <row r="9">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>8172.870000000001</v>
+        <v>204.74</v>
       </c>
     </row>
     <row r="10">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>8748.59</v>
+        <v>151.66</v>
       </c>
     </row>
     <row r="11">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>11597.95</v>
+        <v>133.81</v>
       </c>
     </row>
     <row r="12">
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>9553.629999999999</v>
+        <v>313.86</v>
       </c>
     </row>
     <row r="13">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>94157.60999999999</v>
+        <v>1825.99</v>
       </c>
     </row>
     <row r="15">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>29136.6</v>
+        <v>548.41</v>
       </c>
     </row>
     <row r="17">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>5402</v>
+        <v>122.76</v>
       </c>
     </row>
     <row r="18">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>10899.41</v>
+        <v>201.83</v>
       </c>
     </row>
     <row r="19">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>7979.389999999999</v>
+        <v>252.86</v>
       </c>
     </row>
     <row r="20">
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>22778.60000000001</v>
+        <v>666.6799999999999</v>
       </c>
     </row>
     <row r="21">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>76196</v>
+        <v>1792.54</v>
       </c>
     </row>
     <row r="23">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>5622.52</v>
+        <v>55.76000000000001</v>
       </c>
     </row>
     <row r="25">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>9385.91</v>
+        <v>98.94</v>
       </c>
     </row>
     <row r="26">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>6850.969999999999</v>
+        <v>93.55000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>8356.820000000003</v>
+        <v>92.56</v>
       </c>
     </row>
     <row r="28">
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>29335.50000000001</v>
+        <v>858.1999999999999</v>
       </c>
     </row>
     <row r="29">
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>6715.990000000001</v>
+        <v>106.52</v>
       </c>
     </row>
     <row r="30">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>8493.5</v>
+        <v>108.02</v>
       </c>
     </row>
     <row r="31">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>9704.750000000002</v>
+        <v>218.83</v>
       </c>
     </row>
     <row r="32">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>13555.9</v>
+        <v>560.64</v>
       </c>
     </row>
     <row r="33">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>98021.86000000002</v>
+        <v>2193.02</v>
       </c>
     </row>
     <row r="35">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="B35" s="10" t="n">
-        <v>268375.47</v>
+        <v>5811.55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>